<commit_message>
Fixed issue with one of the isolator footprint names
</commit_message>
<xml_diff>
--- a/To Add v2/Isolators - Digital.xlsx
+++ b/To Add v2/Isolators - Digital.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A4F743C-9B1B-4E6D-8A14-EC4CB5CACD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC74076A-E6CA-46CB-BE37-1D2B66B7B283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>